<commit_message>
Merge color-variant duplicate products in other collections (cross-collection pass)
Cross-collection validation pass found one genuine duplicate: Zenith
Collections' Single Lever Basin Mixer was listed three times (Chrome,
Matt Beige, Matt Black) as separate product groups. Merged into one
group (zenith-collections-001) with a 3-finish picker, following the
same finish-variant merge mechanics and row-ordering fix used for the
Opell Prima merge.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product catalogue.xlsx
+++ b/product catalogue.xlsx
@@ -15362,13 +15362,13 @@
         <v>ZENITH-COLLECTIONS-001</v>
       </c>
       <c r="D300" t="str">
-        <v>Single Lever Basin Mixer Chrome</v>
+        <v>Single Lever Basin Mixer</v>
       </c>
       <c r="E300" t="str">
         <v>Faucets</v>
       </c>
       <c r="F300" t="str">
-        <v/>
+        <v>Chrome</v>
       </c>
       <c r="G300" t="str">
         <v/>
@@ -15406,19 +15406,19 @@
         <v>Zenith Collections</v>
       </c>
       <c r="B301" t="str">
-        <v>zenith-collections-002</v>
+        <v>zenith-collections-001</v>
       </c>
       <c r="C301" t="str">
         <v>ZENITH-COLLECTIONS-002</v>
       </c>
       <c r="D301" t="str">
-        <v>Single Lever Basin Mixer Matt Beige</v>
+        <v/>
       </c>
       <c r="E301" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F301" t="str">
-        <v/>
+        <v>Matt Beige</v>
       </c>
       <c r="G301" t="str">
         <v/>
@@ -15456,19 +15456,19 @@
         <v>Zenith Collections</v>
       </c>
       <c r="B302" t="str">
-        <v>zenith-collections-003</v>
+        <v>zenith-collections-001</v>
       </c>
       <c r="C302" t="str">
         <v>ZENITH-COLLECTIONS-003</v>
       </c>
       <c r="D302" t="str">
-        <v>Single Lever Basin Mixer Matt Black</v>
+        <v/>
       </c>
       <c r="E302" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F302" t="str">
-        <v/>
+        <v>Matt Black</v>
       </c>
       <c r="G302" t="str">
         <v/>

</xml_diff>

<commit_message>
Merge Opell Prima basin mixer color-variant duplicates (006-009)
OPELL-PRIMA-006/007/008/009 were the same wall-mounted basin mixer
upper-part assembly photographed in four finishes (Matt Black Gold,
Matt White Gold, Matt Beige Gold, Matt White) under inconsistent
scraped names. Merged into opell-prima-006 as a single product page
with a 4-finish picker; 49 -> 46 Opell Prima product groups.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product catalogue.xlsx
+++ b/product catalogue.xlsx
@@ -3762,13 +3762,13 @@
         <v>OPELL-PRIMA-006</v>
       </c>
       <c r="D68" t="str">
-        <v>Basin Mixer Upper Part</v>
+        <v>Basin Mixer Wall Mounted Upper Parts</v>
       </c>
       <c r="E68" t="str">
         <v>Faucets</v>
       </c>
       <c r="F68" t="str">
-        <v/>
+        <v>Matt Black Gold</v>
       </c>
       <c r="G68" t="str">
         <v/>
@@ -3806,19 +3806,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B69" t="str">
-        <v>opell-prima-007</v>
+        <v>opell-prima-006</v>
       </c>
       <c r="C69" t="str">
         <v>OPELL-PRIMA-007</v>
       </c>
       <c r="D69" t="str">
-        <v>Basin Mixer Upper Parts</v>
+        <v/>
       </c>
       <c r="E69" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F69" t="str">
-        <v/>
+        <v>Matt White Gold</v>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -3856,19 +3856,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B70" t="str">
-        <v>opell-prima-008</v>
+        <v>opell-prima-006</v>
       </c>
       <c r="C70" t="str">
         <v>OPELL-PRIMA-008</v>
       </c>
       <c r="D70" t="str">
-        <v>Basin Mixer Wall Mounted</v>
+        <v/>
       </c>
       <c r="E70" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F70" t="str">
-        <v/>
+        <v>Matt Beige Gold</v>
       </c>
       <c r="G70" t="str">
         <v/>
@@ -3906,19 +3906,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B71" t="str">
-        <v>opell-prima-009</v>
+        <v>opell-prima-006</v>
       </c>
       <c r="C71" t="str">
         <v>OPELL-PRIMA-009</v>
       </c>
       <c r="D71" t="str">
-        <v>Basin Mixer Wall Mounted Upper Parts</v>
+        <v/>
       </c>
       <c r="E71" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F71" t="str">
-        <v/>
+        <v>Matt White</v>
       </c>
       <c r="G71" t="str">
         <v/>

</xml_diff>

<commit_message>
Merge OPELL-PRIMA-058 (Chrome) into opell-prima-006 as default finish
Chrome is the same wall-mounted basin mixer assembly as the existing
opell-prima-006 group (now 5 finishes: Chrome, Matt Black Gold, Matt
White Gold, Matt Beige Gold, Matt White), with Chrome shown first/by
default on the product and collection pages.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product catalogue.xlsx
+++ b/product catalogue.xlsx
@@ -3759,7 +3759,7 @@
         <v>opell-prima-006</v>
       </c>
       <c r="C68" t="str">
-        <v>OPELL-PRIMA-006</v>
+        <v>OPELL-PRIMA-058</v>
       </c>
       <c r="D68" t="str">
         <v>Basin Mixer Wall Mounted Upper Parts</v>
@@ -3768,7 +3768,7 @@
         <v>Faucets</v>
       </c>
       <c r="F68" t="str">
-        <v>Matt Black Gold</v>
+        <v>Chrome</v>
       </c>
       <c r="G68" t="str">
         <v/>
@@ -3777,7 +3777,7 @@
         <v/>
       </c>
       <c r="I68" t="str">
-        <v>opell-prima-006-main.png</v>
+        <v>opell-prima-058-main.jpg</v>
       </c>
       <c r="J68" t="str">
         <v/>
@@ -3809,7 +3809,7 @@
         <v>opell-prima-006</v>
       </c>
       <c r="C69" t="str">
-        <v>OPELL-PRIMA-007</v>
+        <v>OPELL-PRIMA-006</v>
       </c>
       <c r="D69" t="str">
         <v/>
@@ -3818,7 +3818,7 @@
         <v/>
       </c>
       <c r="F69" t="str">
-        <v>Matt White Gold</v>
+        <v>Matt Black Gold</v>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -3827,7 +3827,7 @@
         <v/>
       </c>
       <c r="I69" t="str">
-        <v>opell-prima-007-main.png</v>
+        <v>opell-prima-006-main.png</v>
       </c>
       <c r="J69" t="str">
         <v/>
@@ -3859,7 +3859,7 @@
         <v>opell-prima-006</v>
       </c>
       <c r="C70" t="str">
-        <v>OPELL-PRIMA-008</v>
+        <v>OPELL-PRIMA-007</v>
       </c>
       <c r="D70" t="str">
         <v/>
@@ -3868,7 +3868,7 @@
         <v/>
       </c>
       <c r="F70" t="str">
-        <v>Matt Beige Gold</v>
+        <v>Matt White Gold</v>
       </c>
       <c r="G70" t="str">
         <v/>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="I70" t="str">
-        <v>opell-prima-008-main.png</v>
+        <v>opell-prima-007-main.png</v>
       </c>
       <c r="J70" t="str">
         <v/>
@@ -3909,7 +3909,7 @@
         <v>opell-prima-006</v>
       </c>
       <c r="C71" t="str">
-        <v>OPELL-PRIMA-009</v>
+        <v>OPELL-PRIMA-008</v>
       </c>
       <c r="D71" t="str">
         <v/>
@@ -3918,7 +3918,7 @@
         <v/>
       </c>
       <c r="F71" t="str">
-        <v>Matt White</v>
+        <v>Matt Beige Gold</v>
       </c>
       <c r="G71" t="str">
         <v/>
@@ -3927,7 +3927,7 @@
         <v/>
       </c>
       <c r="I71" t="str">
-        <v>opell-prima-009-main.png</v>
+        <v>opell-prima-008-main.png</v>
       </c>
       <c r="J71" t="str">
         <v/>
@@ -3956,19 +3956,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B72" t="str">
-        <v>opell-prima-010</v>
+        <v>opell-prima-006</v>
       </c>
       <c r="C72" t="str">
-        <v>OPELL-PRIMA-010</v>
+        <v>OPELL-PRIMA-009</v>
       </c>
       <c r="D72" t="str">
-        <v>Bath TUB Spout</v>
+        <v/>
       </c>
       <c r="E72" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F72" t="str">
-        <v/>
+        <v>Matt White</v>
       </c>
       <c r="G72" t="str">
         <v/>
@@ -3977,7 +3977,7 @@
         <v/>
       </c>
       <c r="I72" t="str">
-        <v>opell-prima-010-main.jpg</v>
+        <v>opell-prima-009-main.png</v>
       </c>
       <c r="J72" t="str">
         <v/>
@@ -4006,16 +4006,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B73" t="str">
-        <v>opell-prima-015</v>
+        <v>opell-prima-010</v>
       </c>
       <c r="C73" t="str">
-        <v>OPELL-PRIMA-015</v>
+        <v>OPELL-PRIMA-010</v>
       </c>
       <c r="D73" t="str">
-        <v>Bottle Trap</v>
+        <v>Bath TUB Spout</v>
       </c>
       <c r="E73" t="str">
-        <v>Accessories</v>
+        <v>Faucets</v>
       </c>
       <c r="F73" t="str">
         <v/>
@@ -4027,7 +4027,7 @@
         <v/>
       </c>
       <c r="I73" t="str">
-        <v>opell-prima-015-main.png</v>
+        <v>opell-prima-010-main.jpg</v>
       </c>
       <c r="J73" t="str">
         <v/>
@@ -4059,16 +4059,16 @@
         <v>opell-prima-015</v>
       </c>
       <c r="C74" t="str">
-        <v>OPELL-PRIMA-011</v>
+        <v>OPELL-PRIMA-015</v>
       </c>
       <c r="D74" t="str">
-        <v/>
+        <v>Bottle Trap</v>
       </c>
       <c r="E74" t="str">
-        <v/>
+        <v>Accessories</v>
       </c>
       <c r="F74" t="str">
-        <v>Matt Beige</v>
+        <v/>
       </c>
       <c r="G74" t="str">
         <v/>
@@ -4077,7 +4077,7 @@
         <v/>
       </c>
       <c r="I74" t="str">
-        <v>opell-prima-011-main.png</v>
+        <v>opell-prima-015-main.png</v>
       </c>
       <c r="J74" t="str">
         <v/>
@@ -4109,7 +4109,7 @@
         <v>opell-prima-015</v>
       </c>
       <c r="C75" t="str">
-        <v>OPELL-PRIMA-014</v>
+        <v>OPELL-PRIMA-011</v>
       </c>
       <c r="D75" t="str">
         <v/>
@@ -4118,7 +4118,7 @@
         <v/>
       </c>
       <c r="F75" t="str">
-        <v>Matt Black</v>
+        <v>Matt Beige</v>
       </c>
       <c r="G75" t="str">
         <v/>
@@ -4127,7 +4127,7 @@
         <v/>
       </c>
       <c r="I75" t="str">
-        <v>opell-prima-014-main.png</v>
+        <v>opell-prima-011-main.png</v>
       </c>
       <c r="J75" t="str">
         <v/>
@@ -4159,7 +4159,7 @@
         <v>opell-prima-015</v>
       </c>
       <c r="C76" t="str">
-        <v>OPELL-PRIMA-016</v>
+        <v>OPELL-PRIMA-014</v>
       </c>
       <c r="D76" t="str">
         <v/>
@@ -4168,7 +4168,7 @@
         <v/>
       </c>
       <c r="F76" t="str">
-        <v>Matt White</v>
+        <v>Matt Black</v>
       </c>
       <c r="G76" t="str">
         <v/>
@@ -4177,7 +4177,7 @@
         <v/>
       </c>
       <c r="I76" t="str">
-        <v>opell-prima-016-main.png</v>
+        <v>opell-prima-014-main.png</v>
       </c>
       <c r="J76" t="str">
         <v/>
@@ -4206,19 +4206,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B77" t="str">
-        <v>opell-prima-012</v>
+        <v>opell-prima-015</v>
       </c>
       <c r="C77" t="str">
-        <v>OPELL-PRIMA-012</v>
+        <v>OPELL-PRIMA-016</v>
       </c>
       <c r="D77" t="str">
-        <v>Beige Gold Alive</v>
+        <v/>
       </c>
       <c r="E77" t="str">
-        <v>Accessories</v>
+        <v/>
       </c>
       <c r="F77" t="str">
-        <v/>
+        <v>Matt White</v>
       </c>
       <c r="G77" t="str">
         <v/>
@@ -4227,7 +4227,7 @@
         <v/>
       </c>
       <c r="I77" t="str">
-        <v>opell-prima-012-main.png</v>
+        <v>opell-prima-016-main.png</v>
       </c>
       <c r="J77" t="str">
         <v/>
@@ -4256,16 +4256,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B78" t="str">
-        <v>opell-prima-013</v>
+        <v>opell-prima-012</v>
       </c>
       <c r="C78" t="str">
-        <v>OPELL-PRIMA-013</v>
+        <v>OPELL-PRIMA-012</v>
       </c>
       <c r="D78" t="str">
-        <v>Beige Gold Shower</v>
+        <v>Beige Gold Alive</v>
       </c>
       <c r="E78" t="str">
-        <v>Showers</v>
+        <v>Accessories</v>
       </c>
       <c r="F78" t="str">
         <v/>
@@ -4277,7 +4277,7 @@
         <v/>
       </c>
       <c r="I78" t="str">
-        <v>opell-prima-013-main.png</v>
+        <v>opell-prima-012-main.png</v>
       </c>
       <c r="J78" t="str">
         <v/>
@@ -4306,16 +4306,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B79" t="str">
-        <v>opell-prima-017</v>
+        <v>opell-prima-013</v>
       </c>
       <c r="C79" t="str">
-        <v>OPELL-PRIMA-017</v>
+        <v>OPELL-PRIMA-013</v>
       </c>
       <c r="D79" t="str">
-        <v>Button Spout</v>
+        <v>Beige Gold Shower</v>
       </c>
       <c r="E79" t="str">
-        <v>Faucets</v>
+        <v>Showers</v>
       </c>
       <c r="F79" t="str">
         <v/>
@@ -4327,7 +4327,7 @@
         <v/>
       </c>
       <c r="I79" t="str">
-        <v>opell-prima-017-main.jpg</v>
+        <v>opell-prima-013-main.png</v>
       </c>
       <c r="J79" t="str">
         <v/>
@@ -4356,16 +4356,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B80" t="str">
-        <v>opell-prima-018</v>
+        <v>opell-prima-017</v>
       </c>
       <c r="C80" t="str">
-        <v>OPELL-PRIMA-018</v>
+        <v>OPELL-PRIMA-017</v>
       </c>
       <c r="D80" t="str">
-        <v>Center Hole</v>
+        <v>Button Spout</v>
       </c>
       <c r="E80" t="str">
-        <v>Accessories</v>
+        <v>Faucets</v>
       </c>
       <c r="F80" t="str">
         <v/>
@@ -4377,7 +4377,7 @@
         <v/>
       </c>
       <c r="I80" t="str">
-        <v>opell-prima-018-main.jpg</v>
+        <v>opell-prima-017-main.jpg</v>
       </c>
       <c r="J80" t="str">
         <v/>
@@ -4406,16 +4406,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B81" t="str">
-        <v>opell-prima-019</v>
+        <v>opell-prima-018</v>
       </c>
       <c r="C81" t="str">
-        <v>OPELL-PRIMA-019</v>
+        <v>OPELL-PRIMA-018</v>
       </c>
       <c r="D81" t="str">
-        <v>Concealed Stop Cock</v>
+        <v>Center Hole</v>
       </c>
       <c r="E81" t="str">
-        <v>Faucets</v>
+        <v>Accessories</v>
       </c>
       <c r="F81" t="str">
         <v/>
@@ -4427,7 +4427,7 @@
         <v/>
       </c>
       <c r="I81" t="str">
-        <v>opell-prima-019-main.jpg</v>
+        <v>opell-prima-018-main.jpg</v>
       </c>
       <c r="J81" t="str">
         <v/>
@@ -4456,13 +4456,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B82" t="str">
-        <v>opell-prima-020</v>
+        <v>opell-prima-019</v>
       </c>
       <c r="C82" t="str">
-        <v>OPELL-PRIMA-020</v>
+        <v>OPELL-PRIMA-019</v>
       </c>
       <c r="D82" t="str">
-        <v>Diverter Body</v>
+        <v>Concealed Stop Cock</v>
       </c>
       <c r="E82" t="str">
         <v>Faucets</v>
@@ -4477,7 +4477,7 @@
         <v/>
       </c>
       <c r="I82" t="str">
-        <v>opell-prima-020-main.png</v>
+        <v>opell-prima-019-main.jpg</v>
       </c>
       <c r="J82" t="str">
         <v/>
@@ -4509,16 +4509,16 @@
         <v>opell-prima-020</v>
       </c>
       <c r="C83" t="str">
-        <v>OPELL-PRIMA-022</v>
+        <v>OPELL-PRIMA-020</v>
       </c>
       <c r="D83" t="str">
-        <v/>
+        <v>Diverter Body</v>
       </c>
       <c r="E83" t="str">
-        <v/>
+        <v>Faucets</v>
       </c>
       <c r="F83" t="str">
-        <v>Rich Gold</v>
+        <v/>
       </c>
       <c r="G83" t="str">
         <v/>
@@ -4527,7 +4527,7 @@
         <v/>
       </c>
       <c r="I83" t="str">
-        <v>opell-prima-022-main.png</v>
+        <v>opell-prima-020-main.png</v>
       </c>
       <c r="J83" t="str">
         <v/>
@@ -4559,7 +4559,7 @@
         <v>opell-prima-020</v>
       </c>
       <c r="C84" t="str">
-        <v>OPELL-PRIMA-023</v>
+        <v>OPELL-PRIMA-022</v>
       </c>
       <c r="D84" t="str">
         <v/>
@@ -4568,7 +4568,7 @@
         <v/>
       </c>
       <c r="F84" t="str">
-        <v>Matt Beige</v>
+        <v>Rich Gold</v>
       </c>
       <c r="G84" t="str">
         <v/>
@@ -4577,7 +4577,7 @@
         <v/>
       </c>
       <c r="I84" t="str">
-        <v>opell-prima-023-main.png</v>
+        <v>opell-prima-022-main.png</v>
       </c>
       <c r="J84" t="str">
         <v/>
@@ -4606,19 +4606,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B85" t="str">
-        <v>opell-prima-021</v>
+        <v>opell-prima-020</v>
       </c>
       <c r="C85" t="str">
-        <v>OPELL-PRIMA-021</v>
+        <v>OPELL-PRIMA-023</v>
       </c>
       <c r="D85" t="str">
-        <v>Diverter Body for ALL Colour and Gold Combination</v>
+        <v/>
       </c>
       <c r="E85" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F85" t="str">
-        <v/>
+        <v>Matt Beige</v>
       </c>
       <c r="G85" t="str">
         <v/>
@@ -4627,7 +4627,7 @@
         <v/>
       </c>
       <c r="I85" t="str">
-        <v>opell-prima-021-main.png</v>
+        <v>opell-prima-023-main.png</v>
       </c>
       <c r="J85" t="str">
         <v/>
@@ -4656,13 +4656,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B86" t="str">
-        <v>opell-prima-024</v>
+        <v>opell-prima-021</v>
       </c>
       <c r="C86" t="str">
-        <v>OPELL-PRIMA-024</v>
+        <v>OPELL-PRIMA-021</v>
       </c>
       <c r="D86" t="str">
-        <v>Diverter Upper Part</v>
+        <v>Diverter Body for ALL Colour and Gold Combination</v>
       </c>
       <c r="E86" t="str">
         <v>Faucets</v>
@@ -4677,7 +4677,7 @@
         <v/>
       </c>
       <c r="I86" t="str">
-        <v>opell-prima-024-main.png</v>
+        <v>opell-prima-021-main.png</v>
       </c>
       <c r="J86" t="str">
         <v/>
@@ -4706,13 +4706,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B87" t="str">
-        <v>opell-prima-025</v>
+        <v>opell-prima-024</v>
       </c>
       <c r="C87" t="str">
-        <v>OPELL-PRIMA-025</v>
+        <v>OPELL-PRIMA-024</v>
       </c>
       <c r="D87" t="str">
-        <v>Diverter Upper Parts</v>
+        <v>Diverter Upper Part</v>
       </c>
       <c r="E87" t="str">
         <v>Faucets</v>
@@ -4727,7 +4727,7 @@
         <v/>
       </c>
       <c r="I87" t="str">
-        <v>opell-prima-025-main.png</v>
+        <v>opell-prima-024-main.png</v>
       </c>
       <c r="J87" t="str">
         <v/>
@@ -4756,13 +4756,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B88" t="str">
-        <v>opell-prima-026</v>
+        <v>opell-prima-025</v>
       </c>
       <c r="C88" t="str">
-        <v>OPELL-PRIMA-026</v>
+        <v>OPELL-PRIMA-025</v>
       </c>
       <c r="D88" t="str">
-        <v>Exposed Parts for Single Lever High Flow Diverter Body</v>
+        <v>Diverter Upper Parts</v>
       </c>
       <c r="E88" t="str">
         <v>Faucets</v>
@@ -4777,7 +4777,7 @@
         <v/>
       </c>
       <c r="I88" t="str">
-        <v>opell-prima-026-main.jpg</v>
+        <v>opell-prima-025-main.png</v>
       </c>
       <c r="J88" t="str">
         <v/>
@@ -4806,16 +4806,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B89" t="str">
-        <v>opell-prima-027</v>
+        <v>opell-prima-026</v>
       </c>
       <c r="C89" t="str">
-        <v>OPELL-PRIMA-027</v>
+        <v>OPELL-PRIMA-026</v>
       </c>
       <c r="D89" t="str">
-        <v>Gold</v>
+        <v>Exposed Parts for Single Lever High Flow Diverter Body</v>
       </c>
       <c r="E89" t="str">
-        <v>Accessories</v>
+        <v>Faucets</v>
       </c>
       <c r="F89" t="str">
         <v/>
@@ -4827,7 +4827,7 @@
         <v/>
       </c>
       <c r="I89" t="str">
-        <v>opell-prima-027-main.png</v>
+        <v>opell-prima-026-main.jpg</v>
       </c>
       <c r="J89" t="str">
         <v/>
@@ -4856,16 +4856,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B90" t="str">
-        <v>opell-prima-029</v>
+        <v>opell-prima-027</v>
       </c>
       <c r="C90" t="str">
-        <v>OPELL-PRIMA-029</v>
+        <v>OPELL-PRIMA-027</v>
       </c>
       <c r="D90" t="str">
-        <v>Hand Shower</v>
+        <v>Gold</v>
       </c>
       <c r="E90" t="str">
-        <v>Showers</v>
+        <v>Accessories</v>
       </c>
       <c r="F90" t="str">
         <v/>
@@ -4877,7 +4877,7 @@
         <v/>
       </c>
       <c r="I90" t="str">
-        <v>opell-prima-029-main.png</v>
+        <v>opell-prima-027-main.png</v>
       </c>
       <c r="J90" t="str">
         <v/>
@@ -4909,16 +4909,16 @@
         <v>opell-prima-029</v>
       </c>
       <c r="C91" t="str">
-        <v>OPELL-PRIMA-028</v>
+        <v>OPELL-PRIMA-029</v>
       </c>
       <c r="D91" t="str">
-        <v/>
+        <v>Hand Shower</v>
       </c>
       <c r="E91" t="str">
-        <v/>
+        <v>Showers</v>
       </c>
       <c r="F91" t="str">
-        <v>Rose Gold</v>
+        <v/>
       </c>
       <c r="G91" t="str">
         <v/>
@@ -4927,7 +4927,7 @@
         <v/>
       </c>
       <c r="I91" t="str">
-        <v>opell-prima-028-main.png</v>
+        <v>opell-prima-029-main.png</v>
       </c>
       <c r="J91" t="str">
         <v/>
@@ -4959,7 +4959,7 @@
         <v>opell-prima-029</v>
       </c>
       <c r="C92" t="str">
-        <v>OPELL-PRIMA-030</v>
+        <v>OPELL-PRIMA-028</v>
       </c>
       <c r="D92" t="str">
         <v/>
@@ -4968,7 +4968,7 @@
         <v/>
       </c>
       <c r="F92" t="str">
-        <v>Rich Gold</v>
+        <v>Rose Gold</v>
       </c>
       <c r="G92" t="str">
         <v/>
@@ -4977,7 +4977,7 @@
         <v/>
       </c>
       <c r="I92" t="str">
-        <v>opell-prima-030-main.png</v>
+        <v>opell-prima-028-main.png</v>
       </c>
       <c r="J92" t="str">
         <v/>
@@ -5006,19 +5006,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B93" t="str">
-        <v>opell-prima-031</v>
+        <v>opell-prima-029</v>
       </c>
       <c r="C93" t="str">
-        <v>OPELL-PRIMA-031</v>
+        <v>OPELL-PRIMA-030</v>
       </c>
       <c r="D93" t="str">
-        <v>Health Faucet</v>
+        <v/>
       </c>
       <c r="E93" t="str">
-        <v>Accessories</v>
+        <v/>
       </c>
       <c r="F93" t="str">
-        <v/>
+        <v>Rich Gold</v>
       </c>
       <c r="G93" t="str">
         <v/>
@@ -5027,7 +5027,7 @@
         <v/>
       </c>
       <c r="I93" t="str">
-        <v>opell-prima-031-main.png</v>
+        <v>opell-prima-030-main.png</v>
       </c>
       <c r="J93" t="str">
         <v/>
@@ -5056,16 +5056,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B94" t="str">
-        <v>opell-prima-032</v>
+        <v>opell-prima-031</v>
       </c>
       <c r="C94" t="str">
-        <v>OPELL-PRIMA-032</v>
+        <v>OPELL-PRIMA-031</v>
       </c>
       <c r="D94" t="str">
-        <v>Long Body</v>
+        <v>Health Faucet</v>
       </c>
       <c r="E94" t="str">
-        <v>Faucets</v>
+        <v>Accessories</v>
       </c>
       <c r="F94" t="str">
         <v/>
@@ -5077,7 +5077,7 @@
         <v/>
       </c>
       <c r="I94" t="str">
-        <v>opell-prima-032-main.jpg</v>
+        <v>opell-prima-031-main.png</v>
       </c>
       <c r="J94" t="str">
         <v/>
@@ -5106,16 +5106,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B95" t="str">
-        <v>opell-prima-033</v>
+        <v>opell-prima-032</v>
       </c>
       <c r="C95" t="str">
-        <v>OPELL-PRIMA-033</v>
+        <v>OPELL-PRIMA-032</v>
       </c>
       <c r="D95" t="str">
-        <v>Matte Beige Alive</v>
+        <v>Long Body</v>
       </c>
       <c r="E95" t="str">
-        <v>Accessories</v>
+        <v>Faucets</v>
       </c>
       <c r="F95" t="str">
         <v/>
@@ -5127,7 +5127,7 @@
         <v/>
       </c>
       <c r="I95" t="str">
-        <v>opell-prima-033-main.png</v>
+        <v>opell-prima-032-main.jpg</v>
       </c>
       <c r="J95" t="str">
         <v/>
@@ -5156,16 +5156,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B96" t="str">
-        <v>opell-prima-034</v>
+        <v>opell-prima-033</v>
       </c>
       <c r="C96" t="str">
-        <v>OPELL-PRIMA-034</v>
+        <v>OPELL-PRIMA-033</v>
       </c>
       <c r="D96" t="str">
-        <v>Matte White Shower Head</v>
+        <v>Matte Beige Alive</v>
       </c>
       <c r="E96" t="str">
-        <v>Showers</v>
+        <v>Accessories</v>
       </c>
       <c r="F96" t="str">
         <v/>
@@ -5177,7 +5177,7 @@
         <v/>
       </c>
       <c r="I96" t="str">
-        <v>opell-prima-034-main.png</v>
+        <v>opell-prima-033-main.png</v>
       </c>
       <c r="J96" t="str">
         <v/>
@@ -5206,16 +5206,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B97" t="str">
-        <v>opell-prima-035</v>
+        <v>opell-prima-034</v>
       </c>
       <c r="C97" t="str">
-        <v>OPELL-PRIMA-035</v>
+        <v>OPELL-PRIMA-034</v>
       </c>
       <c r="D97" t="str">
-        <v>NON Telephonic</v>
+        <v>Matte White Shower Head</v>
       </c>
       <c r="E97" t="str">
-        <v>Accessories</v>
+        <v>Showers</v>
       </c>
       <c r="F97" t="str">
         <v/>
@@ -5227,7 +5227,7 @@
         <v/>
       </c>
       <c r="I97" t="str">
-        <v>opell-prima-035-main.jpg</v>
+        <v>opell-prima-034-main.png</v>
       </c>
       <c r="J97" t="str">
         <v/>
@@ -5256,16 +5256,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B98" t="str">
-        <v>opell-prima-036</v>
+        <v>opell-prima-035</v>
       </c>
       <c r="C98" t="str">
-        <v>OPELL-PRIMA-036</v>
+        <v>OPELL-PRIMA-035</v>
       </c>
       <c r="D98" t="str">
-        <v>Nozzle BIB Cock</v>
+        <v>NON Telephonic</v>
       </c>
       <c r="E98" t="str">
-        <v>Faucets</v>
+        <v>Accessories</v>
       </c>
       <c r="F98" t="str">
         <v/>
@@ -5277,7 +5277,7 @@
         <v/>
       </c>
       <c r="I98" t="str">
-        <v>opell-prima-036-main.jpg</v>
+        <v>opell-prima-035-main.jpg</v>
       </c>
       <c r="J98" t="str">
         <v/>
@@ -5306,13 +5306,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B99" t="str">
-        <v>opell-prima-037</v>
+        <v>opell-prima-036</v>
       </c>
       <c r="C99" t="str">
-        <v>OPELL-PRIMA-037</v>
+        <v>OPELL-PRIMA-036</v>
       </c>
       <c r="D99" t="str">
-        <v>Pillar Cock</v>
+        <v>Nozzle BIB Cock</v>
       </c>
       <c r="E99" t="str">
         <v>Faucets</v>
@@ -5327,7 +5327,7 @@
         <v/>
       </c>
       <c r="I99" t="str">
-        <v>opell-prima-037-main.jpg</v>
+        <v>opell-prima-036-main.jpg</v>
       </c>
       <c r="J99" t="str">
         <v/>
@@ -5356,13 +5356,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B100" t="str">
-        <v>opell-prima-038</v>
+        <v>opell-prima-037</v>
       </c>
       <c r="C100" t="str">
-        <v>OPELL-PRIMA-038</v>
+        <v>OPELL-PRIMA-037</v>
       </c>
       <c r="D100" t="str">
-        <v>Pillar Cock Extend</v>
+        <v>Pillar Cock</v>
       </c>
       <c r="E100" t="str">
         <v>Faucets</v>
@@ -5377,7 +5377,7 @@
         <v/>
       </c>
       <c r="I100" t="str">
-        <v>opell-prima-038-main.png</v>
+        <v>opell-prima-037-main.jpg</v>
       </c>
       <c r="J100" t="str">
         <v/>
@@ -5406,13 +5406,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B101" t="str">
-        <v>opell-prima-039</v>
+        <v>opell-prima-038</v>
       </c>
       <c r="C101" t="str">
-        <v>OPELL-PRIMA-039</v>
+        <v>OPELL-PRIMA-038</v>
       </c>
       <c r="D101" t="str">
-        <v>Pillar Cock Extended</v>
+        <v>Pillar Cock Extend</v>
       </c>
       <c r="E101" t="str">
         <v>Faucets</v>
@@ -5427,7 +5427,7 @@
         <v/>
       </c>
       <c r="I101" t="str">
-        <v>opell-prima-039-main.png</v>
+        <v>opell-prima-038-main.png</v>
       </c>
       <c r="J101" t="str">
         <v/>
@@ -5456,13 +5456,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B102" t="str">
-        <v>opell-prima-040</v>
+        <v>opell-prima-039</v>
       </c>
       <c r="C102" t="str">
-        <v>OPELL-PRIMA-040</v>
+        <v>OPELL-PRIMA-039</v>
       </c>
       <c r="D102" t="str">
-        <v>Pillar Cock Extended Body</v>
+        <v>Pillar Cock Extended</v>
       </c>
       <c r="E102" t="str">
         <v>Faucets</v>
@@ -5477,7 +5477,7 @@
         <v/>
       </c>
       <c r="I102" t="str">
-        <v>opell-prima-040-main.jpg</v>
+        <v>opell-prima-039-main.png</v>
       </c>
       <c r="J102" t="str">
         <v/>
@@ -5506,13 +5506,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B103" t="str">
-        <v>opell-prima-041</v>
+        <v>opell-prima-040</v>
       </c>
       <c r="C103" t="str">
-        <v>OPELL-PRIMA-041</v>
+        <v>OPELL-PRIMA-040</v>
       </c>
       <c r="D103" t="str">
-        <v>Plain Spout</v>
+        <v>Pillar Cock Extended Body</v>
       </c>
       <c r="E103" t="str">
         <v>Faucets</v>
@@ -5527,7 +5527,7 @@
         <v/>
       </c>
       <c r="I103" t="str">
-        <v>opell-prima-041-main.png</v>
+        <v>opell-prima-040-main.jpg</v>
       </c>
       <c r="J103" t="str">
         <v/>
@@ -5556,16 +5556,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B104" t="str">
-        <v>opell-prima-042</v>
+        <v>opell-prima-041</v>
       </c>
       <c r="C104" t="str">
-        <v>OPELL-PRIMA-042</v>
+        <v>OPELL-PRIMA-041</v>
       </c>
       <c r="D104" t="str">
-        <v>Shower ARM</v>
+        <v>Plain Spout</v>
       </c>
       <c r="E104" t="str">
-        <v>Showers</v>
+        <v>Faucets</v>
       </c>
       <c r="F104" t="str">
         <v/>
@@ -5577,7 +5577,7 @@
         <v/>
       </c>
       <c r="I104" t="str">
-        <v>opell-prima-042-main.png</v>
+        <v>opell-prima-041-main.png</v>
       </c>
       <c r="J104" t="str">
         <v/>
@@ -5609,16 +5609,16 @@
         <v>opell-prima-042</v>
       </c>
       <c r="C105" t="str">
-        <v>OPELL-PRIMA-043</v>
+        <v>OPELL-PRIMA-042</v>
       </c>
       <c r="D105" t="str">
-        <v/>
+        <v>Shower ARM</v>
       </c>
       <c r="E105" t="str">
-        <v/>
+        <v>Showers</v>
       </c>
       <c r="F105" t="str">
-        <v>Matt Black Gold</v>
+        <v/>
       </c>
       <c r="G105" t="str">
         <v/>
@@ -5627,7 +5627,7 @@
         <v/>
       </c>
       <c r="I105" t="str">
-        <v>opell-prima-043-main.png</v>
+        <v>opell-prima-042-main.png</v>
       </c>
       <c r="J105" t="str">
         <v/>
@@ -5656,19 +5656,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B106" t="str">
-        <v>opell-prima-044</v>
+        <v>opell-prima-042</v>
       </c>
       <c r="C106" t="str">
-        <v>OPELL-PRIMA-044</v>
+        <v>OPELL-PRIMA-043</v>
       </c>
       <c r="D106" t="str">
-        <v>Shower Head</v>
+        <v/>
       </c>
       <c r="E106" t="str">
-        <v>Showers</v>
+        <v/>
       </c>
       <c r="F106" t="str">
-        <v/>
+        <v>Matt Black Gold</v>
       </c>
       <c r="G106" t="str">
         <v/>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="I106" t="str">
-        <v>opell-prima-044-main.png</v>
+        <v>opell-prima-043-main.png</v>
       </c>
       <c r="J106" t="str">
         <v/>
@@ -5709,16 +5709,16 @@
         <v>opell-prima-044</v>
       </c>
       <c r="C107" t="str">
-        <v>OPELL-PRIMA-045</v>
+        <v>OPELL-PRIMA-044</v>
       </c>
       <c r="D107" t="str">
-        <v/>
+        <v>Shower Head</v>
       </c>
       <c r="E107" t="str">
-        <v/>
+        <v>Showers</v>
       </c>
       <c r="F107" t="str">
-        <v>Matt Beige</v>
+        <v/>
       </c>
       <c r="G107" t="str">
         <v/>
@@ -5727,7 +5727,7 @@
         <v/>
       </c>
       <c r="I107" t="str">
-        <v>opell-prima-045-main.png</v>
+        <v>opell-prima-044-main.png</v>
       </c>
       <c r="J107" t="str">
         <v/>
@@ -5756,19 +5756,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B108" t="str">
-        <v>opell-prima-046</v>
+        <v>opell-prima-044</v>
       </c>
       <c r="C108" t="str">
-        <v>OPELL-PRIMA-046</v>
+        <v>OPELL-PRIMA-045</v>
       </c>
       <c r="D108" t="str">
-        <v>Shower Mixer for Spout Only</v>
+        <v/>
       </c>
       <c r="E108" t="str">
-        <v>Showers</v>
+        <v/>
       </c>
       <c r="F108" t="str">
-        <v/>
+        <v>Matt Beige</v>
       </c>
       <c r="G108" t="str">
         <v/>
@@ -5777,7 +5777,7 @@
         <v/>
       </c>
       <c r="I108" t="str">
-        <v>opell-prima-046-main.jpg</v>
+        <v>opell-prima-045-main.png</v>
       </c>
       <c r="J108" t="str">
         <v/>
@@ -5806,16 +5806,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B109" t="str">
-        <v>opell-prima-047</v>
+        <v>opell-prima-046</v>
       </c>
       <c r="C109" t="str">
-        <v>OPELL-PRIMA-047</v>
+        <v>OPELL-PRIMA-046</v>
       </c>
       <c r="D109" t="str">
-        <v>Single Lever Basin Mixer</v>
+        <v>Shower Mixer for Spout Only</v>
       </c>
       <c r="E109" t="str">
-        <v>Faucets</v>
+        <v>Showers</v>
       </c>
       <c r="F109" t="str">
         <v/>
@@ -5827,10 +5827,10 @@
         <v/>
       </c>
       <c r="I109" t="str">
-        <v>opell-prima-047-main.jpg</v>
+        <v>opell-prima-046-main.jpg</v>
       </c>
       <c r="J109" t="str">
-        <v>opell-prima-047-main.jpg,opell-prima-059-main.png</v>
+        <v/>
       </c>
       <c r="K109" t="str">
         <v/>
@@ -5856,13 +5856,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B110" t="str">
-        <v>opell-prima-048</v>
+        <v>opell-prima-047</v>
       </c>
       <c r="C110" t="str">
-        <v>OPELL-PRIMA-048</v>
+        <v>OPELL-PRIMA-047</v>
       </c>
       <c r="D110" t="str">
-        <v>Single Lever Basin Mixer Extended Body</v>
+        <v>Single Lever Basin Mixer</v>
       </c>
       <c r="E110" t="str">
         <v>Faucets</v>
@@ -5877,10 +5877,10 @@
         <v/>
       </c>
       <c r="I110" t="str">
-        <v>opell-prima-048-main.jpg</v>
+        <v>opell-prima-047-main.jpg</v>
       </c>
       <c r="J110" t="str">
-        <v/>
+        <v>opell-prima-047-main.jpg,opell-prima-059-main.png</v>
       </c>
       <c r="K110" t="str">
         <v/>
@@ -5906,13 +5906,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B111" t="str">
-        <v>opell-prima-049</v>
+        <v>opell-prima-048</v>
       </c>
       <c r="C111" t="str">
-        <v>OPELL-PRIMA-049</v>
+        <v>OPELL-PRIMA-048</v>
       </c>
       <c r="D111" t="str">
-        <v>Single Lever Basin Mixer Tall</v>
+        <v>Single Lever Basin Mixer Extended Body</v>
       </c>
       <c r="E111" t="str">
         <v>Faucets</v>
@@ -5927,10 +5927,10 @@
         <v/>
       </c>
       <c r="I111" t="str">
-        <v>opell-prima-049-main.png</v>
+        <v>opell-prima-048-main.jpg</v>
       </c>
       <c r="J111" t="str">
-        <v>opell-prima-049-main.png,opell-prima-060-main.png</v>
+        <v/>
       </c>
       <c r="K111" t="str">
         <v/>
@@ -5956,16 +5956,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B112" t="str">
-        <v>opell-prima-050</v>
+        <v>opell-prima-049</v>
       </c>
       <c r="C112" t="str">
-        <v>OPELL-PRIMA-050</v>
+        <v>OPELL-PRIMA-049</v>
       </c>
       <c r="D112" t="str">
-        <v>Single Lever Basin Tall</v>
+        <v>Single Lever Basin Mixer Tall</v>
       </c>
       <c r="E112" t="str">
-        <v>Accessories</v>
+        <v>Faucets</v>
       </c>
       <c r="F112" t="str">
         <v/>
@@ -5977,10 +5977,10 @@
         <v/>
       </c>
       <c r="I112" t="str">
-        <v>opell-prima-050-main.png</v>
+        <v>opell-prima-049-main.png</v>
       </c>
       <c r="J112" t="str">
-        <v/>
+        <v>opell-prima-049-main.png,opell-prima-060-main.png</v>
       </c>
       <c r="K112" t="str">
         <v/>
@@ -6006,16 +6006,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B113" t="str">
-        <v>opell-prima-051</v>
+        <v>opell-prima-050</v>
       </c>
       <c r="C113" t="str">
-        <v>OPELL-PRIMA-051</v>
+        <v>OPELL-PRIMA-050</v>
       </c>
       <c r="D113" t="str">
-        <v>Single Lever Exposed Shower Mixer</v>
+        <v>Single Lever Basin Tall</v>
       </c>
       <c r="E113" t="str">
-        <v>Showers</v>
+        <v>Accessories</v>
       </c>
       <c r="F113" t="str">
         <v/>
@@ -6027,7 +6027,7 @@
         <v/>
       </c>
       <c r="I113" t="str">
-        <v>opell-prima-051-main.jpg</v>
+        <v>opell-prima-050-main.png</v>
       </c>
       <c r="J113" t="str">
         <v/>
@@ -6056,16 +6056,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B114" t="str">
-        <v>opell-prima-052</v>
+        <v>opell-prima-051</v>
       </c>
       <c r="C114" t="str">
-        <v>OPELL-PRIMA-052</v>
+        <v>OPELL-PRIMA-051</v>
       </c>
       <c r="D114" t="str">
-        <v>Single Lever Sink Mixer Table Mounted Angular Spout</v>
+        <v>Single Lever Exposed Shower Mixer</v>
       </c>
       <c r="E114" t="str">
-        <v>Faucets</v>
+        <v>Showers</v>
       </c>
       <c r="F114" t="str">
         <v/>
@@ -6077,7 +6077,7 @@
         <v/>
       </c>
       <c r="I114" t="str">
-        <v>opell-prima-052-main.jpg</v>
+        <v>opell-prima-051-main.jpg</v>
       </c>
       <c r="J114" t="str">
         <v/>
@@ -6106,13 +6106,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B115" t="str">
-        <v>opell-prima-053</v>
+        <v>opell-prima-052</v>
       </c>
       <c r="C115" t="str">
-        <v>OPELL-PRIMA-053</v>
+        <v>OPELL-PRIMA-052</v>
       </c>
       <c r="D115" t="str">
-        <v>Single Lever Sink Mixer Table Mounted Round Spout Side Handle</v>
+        <v>Single Lever Sink Mixer Table Mounted Angular Spout</v>
       </c>
       <c r="E115" t="str">
         <v>Faucets</v>
@@ -6127,7 +6127,7 @@
         <v/>
       </c>
       <c r="I115" t="str">
-        <v>opell-prima-053-main.jpg</v>
+        <v>opell-prima-052-main.jpg</v>
       </c>
       <c r="J115" t="str">
         <v/>
@@ -6156,13 +6156,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B116" t="str">
-        <v>opell-prima-054</v>
+        <v>opell-prima-053</v>
       </c>
       <c r="C116" t="str">
-        <v>OPELL-PRIMA-054</v>
+        <v>OPELL-PRIMA-053</v>
       </c>
       <c r="D116" t="str">
-        <v>Single Lever Sink Mixer Table Mounted Tall</v>
+        <v>Single Lever Sink Mixer Table Mounted Round Spout Side Handle</v>
       </c>
       <c r="E116" t="str">
         <v>Faucets</v>
@@ -6177,7 +6177,7 @@
         <v/>
       </c>
       <c r="I116" t="str">
-        <v>opell-prima-054-main.jpg</v>
+        <v>opell-prima-053-main.jpg</v>
       </c>
       <c r="J116" t="str">
         <v/>
@@ -6206,13 +6206,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B117" t="str">
-        <v>opell-prima-055</v>
+        <v>opell-prima-054</v>
       </c>
       <c r="C117" t="str">
-        <v>OPELL-PRIMA-055</v>
+        <v>OPELL-PRIMA-054</v>
       </c>
       <c r="D117" t="str">
-        <v>Single Lever Sink Mixer Wall Mounted Angular Spout</v>
+        <v>Single Lever Sink Mixer Table Mounted Tall</v>
       </c>
       <c r="E117" t="str">
         <v>Faucets</v>
@@ -6227,7 +6227,7 @@
         <v/>
       </c>
       <c r="I117" t="str">
-        <v>opell-prima-055-main.jpg</v>
+        <v>opell-prima-054-main.jpg</v>
       </c>
       <c r="J117" t="str">
         <v/>
@@ -6256,13 +6256,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B118" t="str">
-        <v>opell-prima-056</v>
+        <v>opell-prima-055</v>
       </c>
       <c r="C118" t="str">
-        <v>OPELL-PRIMA-056</v>
+        <v>OPELL-PRIMA-055</v>
       </c>
       <c r="D118" t="str">
-        <v>Single Lever Sink Mixer Wall Mounted Round Spout</v>
+        <v>Single Lever Sink Mixer Wall Mounted Angular Spout</v>
       </c>
       <c r="E118" t="str">
         <v>Faucets</v>
@@ -6277,7 +6277,7 @@
         <v/>
       </c>
       <c r="I118" t="str">
-        <v>opell-prima-056-main.jpg</v>
+        <v>opell-prima-055-main.jpg</v>
       </c>
       <c r="J118" t="str">
         <v/>
@@ -6306,13 +6306,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B119" t="str">
-        <v>opell-prima-057</v>
+        <v>opell-prima-056</v>
       </c>
       <c r="C119" t="str">
-        <v>OPELL-PRIMA-057</v>
+        <v>OPELL-PRIMA-056</v>
       </c>
       <c r="D119" t="str">
-        <v>Single Lever Wall Mixer</v>
+        <v>Single Lever Sink Mixer Wall Mounted Round Spout</v>
       </c>
       <c r="E119" t="str">
         <v>Faucets</v>
@@ -6327,7 +6327,7 @@
         <v/>
       </c>
       <c r="I119" t="str">
-        <v>opell-prima-057-main.jpg</v>
+        <v>opell-prima-056-main.jpg</v>
       </c>
       <c r="J119" t="str">
         <v/>
@@ -6356,13 +6356,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B120" t="str">
-        <v>opell-prima-058</v>
+        <v>opell-prima-057</v>
       </c>
       <c r="C120" t="str">
-        <v>OPELL-PRIMA-058</v>
+        <v>OPELL-PRIMA-057</v>
       </c>
       <c r="D120" t="str">
-        <v>Single Lever Wall Mounted Basin Mixer</v>
+        <v>Single Lever Wall Mixer</v>
       </c>
       <c r="E120" t="str">
         <v>Faucets</v>
@@ -6377,7 +6377,7 @@
         <v/>
       </c>
       <c r="I120" t="str">
-        <v>opell-prima-058-main.jpg</v>
+        <v>opell-prima-057-main.jpg</v>
       </c>
       <c r="J120" t="str">
         <v/>

</xml_diff>

<commit_message>
Merge 3 more Opell Prima color-variant duplicate groups
- OPELL-PRIMA-003/012/033 (Aliva Shower Head): Chrome, Profile Beige
  Gold, Matt Beige
- OPELL-PRIMA-024/025/026 (Diverter upper parts): Matt Black, Rich
  Gold, Chrome
- OPELL-PRIMA-038/039/048/049/050 (Tall single lever basin mixer):
  Matt Beige, Rose Gold, Chrome, Matt White, Matt Beige Gold

Opell Prima groups: 45 -> 37, product pages: 298 -> 290.

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/product catalogue.xlsx
+++ b/product catalogue.xlsx
@@ -3668,7 +3668,7 @@
         <v>Showers</v>
       </c>
       <c r="F66" t="str">
-        <v/>
+        <v>Chrome</v>
       </c>
       <c r="G66" t="str">
         <v/>
@@ -3706,19 +3706,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B67" t="str">
-        <v>opell-prima-005</v>
+        <v>opell-prima-003</v>
       </c>
       <c r="C67" t="str">
-        <v>OPELL-PRIMA-005</v>
+        <v>OPELL-PRIMA-012</v>
       </c>
       <c r="D67" t="str">
-        <v>Angle Valve</v>
+        <v/>
       </c>
       <c r="E67" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F67" t="str">
-        <v/>
+        <v>Profile Beige Gold</v>
       </c>
       <c r="G67" t="str">
         <v/>
@@ -3727,7 +3727,7 @@
         <v/>
       </c>
       <c r="I67" t="str">
-        <v>opell-prima-005-main.jpg</v>
+        <v>opell-prima-012-main.png</v>
       </c>
       <c r="J67" t="str">
         <v/>
@@ -3756,19 +3756,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B68" t="str">
-        <v>opell-prima-006</v>
+        <v>opell-prima-003</v>
       </c>
       <c r="C68" t="str">
-        <v>OPELL-PRIMA-058</v>
+        <v>OPELL-PRIMA-033</v>
       </c>
       <c r="D68" t="str">
-        <v>Basin Mixer Wall Mounted Upper Parts</v>
+        <v/>
       </c>
       <c r="E68" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F68" t="str">
-        <v>Chrome</v>
+        <v>Matt Beige</v>
       </c>
       <c r="G68" t="str">
         <v/>
@@ -3777,7 +3777,7 @@
         <v/>
       </c>
       <c r="I68" t="str">
-        <v>opell-prima-058-main.jpg</v>
+        <v>opell-prima-033-main.png</v>
       </c>
       <c r="J68" t="str">
         <v/>
@@ -3806,19 +3806,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B69" t="str">
-        <v>opell-prima-006</v>
+        <v>opell-prima-005</v>
       </c>
       <c r="C69" t="str">
-        <v>OPELL-PRIMA-006</v>
+        <v>OPELL-PRIMA-005</v>
       </c>
       <c r="D69" t="str">
-        <v/>
+        <v>Angle Valve</v>
       </c>
       <c r="E69" t="str">
-        <v/>
+        <v>Faucets</v>
       </c>
       <c r="F69" t="str">
-        <v>Matt Black Gold</v>
+        <v/>
       </c>
       <c r="G69" t="str">
         <v/>
@@ -3827,7 +3827,7 @@
         <v/>
       </c>
       <c r="I69" t="str">
-        <v>opell-prima-006-main.png</v>
+        <v>opell-prima-005-main.jpg</v>
       </c>
       <c r="J69" t="str">
         <v/>
@@ -3859,16 +3859,16 @@
         <v>opell-prima-006</v>
       </c>
       <c r="C70" t="str">
-        <v>OPELL-PRIMA-007</v>
+        <v>OPELL-PRIMA-058</v>
       </c>
       <c r="D70" t="str">
-        <v/>
+        <v>Basin Mixer Wall Mounted Upper Parts</v>
       </c>
       <c r="E70" t="str">
-        <v/>
+        <v>Faucets</v>
       </c>
       <c r="F70" t="str">
-        <v>Matt White Gold</v>
+        <v>Chrome</v>
       </c>
       <c r="G70" t="str">
         <v/>
@@ -3877,7 +3877,7 @@
         <v/>
       </c>
       <c r="I70" t="str">
-        <v>opell-prima-007-main.png</v>
+        <v>opell-prima-058-main.jpg</v>
       </c>
       <c r="J70" t="str">
         <v/>
@@ -3909,7 +3909,7 @@
         <v>opell-prima-006</v>
       </c>
       <c r="C71" t="str">
-        <v>OPELL-PRIMA-008</v>
+        <v>OPELL-PRIMA-006</v>
       </c>
       <c r="D71" t="str">
         <v/>
@@ -3918,7 +3918,7 @@
         <v/>
       </c>
       <c r="F71" t="str">
-        <v>Matt Beige Gold</v>
+        <v>Matt Black Gold</v>
       </c>
       <c r="G71" t="str">
         <v/>
@@ -3927,7 +3927,7 @@
         <v/>
       </c>
       <c r="I71" t="str">
-        <v>opell-prima-008-main.png</v>
+        <v>opell-prima-006-main.png</v>
       </c>
       <c r="J71" t="str">
         <v/>
@@ -3959,7 +3959,7 @@
         <v>opell-prima-006</v>
       </c>
       <c r="C72" t="str">
-        <v>OPELL-PRIMA-009</v>
+        <v>OPELL-PRIMA-007</v>
       </c>
       <c r="D72" t="str">
         <v/>
@@ -3968,7 +3968,7 @@
         <v/>
       </c>
       <c r="F72" t="str">
-        <v>Matt White</v>
+        <v>Matt White Gold</v>
       </c>
       <c r="G72" t="str">
         <v/>
@@ -3977,7 +3977,7 @@
         <v/>
       </c>
       <c r="I72" t="str">
-        <v>opell-prima-009-main.png</v>
+        <v>opell-prima-007-main.png</v>
       </c>
       <c r="J72" t="str">
         <v/>
@@ -4006,19 +4006,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B73" t="str">
-        <v>opell-prima-010</v>
+        <v>opell-prima-006</v>
       </c>
       <c r="C73" t="str">
-        <v>OPELL-PRIMA-010</v>
+        <v>OPELL-PRIMA-008</v>
       </c>
       <c r="D73" t="str">
-        <v>Bath TUB Spout</v>
+        <v/>
       </c>
       <c r="E73" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F73" t="str">
-        <v/>
+        <v>Matt Beige Gold</v>
       </c>
       <c r="G73" t="str">
         <v/>
@@ -4027,7 +4027,7 @@
         <v/>
       </c>
       <c r="I73" t="str">
-        <v>opell-prima-010-main.jpg</v>
+        <v>opell-prima-008-main.png</v>
       </c>
       <c r="J73" t="str">
         <v/>
@@ -4056,19 +4056,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B74" t="str">
-        <v>opell-prima-015</v>
+        <v>opell-prima-006</v>
       </c>
       <c r="C74" t="str">
-        <v>OPELL-PRIMA-015</v>
+        <v>OPELL-PRIMA-009</v>
       </c>
       <c r="D74" t="str">
-        <v>Bottle Trap</v>
+        <v/>
       </c>
       <c r="E74" t="str">
-        <v>Accessories</v>
+        <v/>
       </c>
       <c r="F74" t="str">
-        <v/>
+        <v>Matt White</v>
       </c>
       <c r="G74" t="str">
         <v/>
@@ -4077,7 +4077,7 @@
         <v/>
       </c>
       <c r="I74" t="str">
-        <v>opell-prima-015-main.png</v>
+        <v>opell-prima-009-main.png</v>
       </c>
       <c r="J74" t="str">
         <v/>
@@ -4106,19 +4106,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B75" t="str">
-        <v>opell-prima-015</v>
+        <v>opell-prima-010</v>
       </c>
       <c r="C75" t="str">
-        <v>OPELL-PRIMA-011</v>
+        <v>OPELL-PRIMA-010</v>
       </c>
       <c r="D75" t="str">
-        <v/>
+        <v>Bath TUB Spout</v>
       </c>
       <c r="E75" t="str">
-        <v/>
+        <v>Faucets</v>
       </c>
       <c r="F75" t="str">
-        <v>Matt Beige</v>
+        <v/>
       </c>
       <c r="G75" t="str">
         <v/>
@@ -4127,7 +4127,7 @@
         <v/>
       </c>
       <c r="I75" t="str">
-        <v>opell-prima-011-main.png</v>
+        <v>opell-prima-010-main.jpg</v>
       </c>
       <c r="J75" t="str">
         <v/>
@@ -4159,16 +4159,16 @@
         <v>opell-prima-015</v>
       </c>
       <c r="C76" t="str">
-        <v>OPELL-PRIMA-014</v>
+        <v>OPELL-PRIMA-015</v>
       </c>
       <c r="D76" t="str">
-        <v/>
+        <v>Bottle Trap</v>
       </c>
       <c r="E76" t="str">
-        <v/>
+        <v>Accessories</v>
       </c>
       <c r="F76" t="str">
-        <v>Matt Black</v>
+        <v/>
       </c>
       <c r="G76" t="str">
         <v/>
@@ -4177,7 +4177,7 @@
         <v/>
       </c>
       <c r="I76" t="str">
-        <v>opell-prima-014-main.png</v>
+        <v>opell-prima-015-main.png</v>
       </c>
       <c r="J76" t="str">
         <v/>
@@ -4209,7 +4209,7 @@
         <v>opell-prima-015</v>
       </c>
       <c r="C77" t="str">
-        <v>OPELL-PRIMA-016</v>
+        <v>OPELL-PRIMA-011</v>
       </c>
       <c r="D77" t="str">
         <v/>
@@ -4218,7 +4218,7 @@
         <v/>
       </c>
       <c r="F77" t="str">
-        <v>Matt White</v>
+        <v>Matt Beige</v>
       </c>
       <c r="G77" t="str">
         <v/>
@@ -4227,7 +4227,7 @@
         <v/>
       </c>
       <c r="I77" t="str">
-        <v>opell-prima-016-main.png</v>
+        <v>opell-prima-011-main.png</v>
       </c>
       <c r="J77" t="str">
         <v/>
@@ -4256,19 +4256,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B78" t="str">
-        <v>opell-prima-012</v>
+        <v>opell-prima-015</v>
       </c>
       <c r="C78" t="str">
-        <v>OPELL-PRIMA-012</v>
+        <v>OPELL-PRIMA-014</v>
       </c>
       <c r="D78" t="str">
-        <v>Beige Gold Alive</v>
+        <v/>
       </c>
       <c r="E78" t="str">
-        <v>Accessories</v>
+        <v/>
       </c>
       <c r="F78" t="str">
-        <v/>
+        <v>Matt Black</v>
       </c>
       <c r="G78" t="str">
         <v/>
@@ -4277,7 +4277,7 @@
         <v/>
       </c>
       <c r="I78" t="str">
-        <v>opell-prima-012-main.png</v>
+        <v>opell-prima-014-main.png</v>
       </c>
       <c r="J78" t="str">
         <v/>
@@ -4306,19 +4306,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B79" t="str">
-        <v>opell-prima-013</v>
+        <v>opell-prima-015</v>
       </c>
       <c r="C79" t="str">
-        <v>OPELL-PRIMA-013</v>
+        <v>OPELL-PRIMA-016</v>
       </c>
       <c r="D79" t="str">
-        <v>Beige Gold Shower</v>
+        <v/>
       </c>
       <c r="E79" t="str">
-        <v>Showers</v>
+        <v/>
       </c>
       <c r="F79" t="str">
-        <v/>
+        <v>Matt White</v>
       </c>
       <c r="G79" t="str">
         <v/>
@@ -4327,7 +4327,7 @@
         <v/>
       </c>
       <c r="I79" t="str">
-        <v>opell-prima-013-main.png</v>
+        <v>opell-prima-016-main.png</v>
       </c>
       <c r="J79" t="str">
         <v/>
@@ -4356,16 +4356,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B80" t="str">
-        <v>opell-prima-017</v>
+        <v>opell-prima-013</v>
       </c>
       <c r="C80" t="str">
-        <v>OPELL-PRIMA-017</v>
+        <v>OPELL-PRIMA-013</v>
       </c>
       <c r="D80" t="str">
-        <v>Button Spout</v>
+        <v>Beige Gold Shower</v>
       </c>
       <c r="E80" t="str">
-        <v>Faucets</v>
+        <v>Showers</v>
       </c>
       <c r="F80" t="str">
         <v/>
@@ -4377,7 +4377,7 @@
         <v/>
       </c>
       <c r="I80" t="str">
-        <v>opell-prima-017-main.jpg</v>
+        <v>opell-prima-013-main.png</v>
       </c>
       <c r="J80" t="str">
         <v/>
@@ -4406,16 +4406,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B81" t="str">
-        <v>opell-prima-018</v>
+        <v>opell-prima-017</v>
       </c>
       <c r="C81" t="str">
-        <v>OPELL-PRIMA-018</v>
+        <v>OPELL-PRIMA-017</v>
       </c>
       <c r="D81" t="str">
-        <v>Center Hole</v>
+        <v>Button Spout</v>
       </c>
       <c r="E81" t="str">
-        <v>Accessories</v>
+        <v>Faucets</v>
       </c>
       <c r="F81" t="str">
         <v/>
@@ -4427,7 +4427,7 @@
         <v/>
       </c>
       <c r="I81" t="str">
-        <v>opell-prima-018-main.jpg</v>
+        <v>opell-prima-017-main.jpg</v>
       </c>
       <c r="J81" t="str">
         <v/>
@@ -4456,16 +4456,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B82" t="str">
-        <v>opell-prima-019</v>
+        <v>opell-prima-018</v>
       </c>
       <c r="C82" t="str">
-        <v>OPELL-PRIMA-019</v>
+        <v>OPELL-PRIMA-018</v>
       </c>
       <c r="D82" t="str">
-        <v>Concealed Stop Cock</v>
+        <v>Center Hole</v>
       </c>
       <c r="E82" t="str">
-        <v>Faucets</v>
+        <v>Accessories</v>
       </c>
       <c r="F82" t="str">
         <v/>
@@ -4477,7 +4477,7 @@
         <v/>
       </c>
       <c r="I82" t="str">
-        <v>opell-prima-019-main.jpg</v>
+        <v>opell-prima-018-main.jpg</v>
       </c>
       <c r="J82" t="str">
         <v/>
@@ -4506,13 +4506,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B83" t="str">
-        <v>opell-prima-020</v>
+        <v>opell-prima-019</v>
       </c>
       <c r="C83" t="str">
-        <v>OPELL-PRIMA-020</v>
+        <v>OPELL-PRIMA-019</v>
       </c>
       <c r="D83" t="str">
-        <v>Diverter Body</v>
+        <v>Concealed Stop Cock</v>
       </c>
       <c r="E83" t="str">
         <v>Faucets</v>
@@ -4527,7 +4527,7 @@
         <v/>
       </c>
       <c r="I83" t="str">
-        <v>opell-prima-020-main.png</v>
+        <v>opell-prima-019-main.jpg</v>
       </c>
       <c r="J83" t="str">
         <v/>
@@ -4559,16 +4559,16 @@
         <v>opell-prima-020</v>
       </c>
       <c r="C84" t="str">
-        <v>OPELL-PRIMA-022</v>
+        <v>OPELL-PRIMA-020</v>
       </c>
       <c r="D84" t="str">
-        <v/>
+        <v>Diverter Body</v>
       </c>
       <c r="E84" t="str">
-        <v/>
+        <v>Faucets</v>
       </c>
       <c r="F84" t="str">
-        <v>Rich Gold</v>
+        <v/>
       </c>
       <c r="G84" t="str">
         <v/>
@@ -4577,7 +4577,7 @@
         <v/>
       </c>
       <c r="I84" t="str">
-        <v>opell-prima-022-main.png</v>
+        <v>opell-prima-020-main.png</v>
       </c>
       <c r="J84" t="str">
         <v/>
@@ -4609,7 +4609,7 @@
         <v>opell-prima-020</v>
       </c>
       <c r="C85" t="str">
-        <v>OPELL-PRIMA-023</v>
+        <v>OPELL-PRIMA-022</v>
       </c>
       <c r="D85" t="str">
         <v/>
@@ -4618,7 +4618,7 @@
         <v/>
       </c>
       <c r="F85" t="str">
-        <v>Matt Beige</v>
+        <v>Rich Gold</v>
       </c>
       <c r="G85" t="str">
         <v/>
@@ -4627,7 +4627,7 @@
         <v/>
       </c>
       <c r="I85" t="str">
-        <v>opell-prima-023-main.png</v>
+        <v>opell-prima-022-main.png</v>
       </c>
       <c r="J85" t="str">
         <v/>
@@ -4656,19 +4656,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B86" t="str">
-        <v>opell-prima-021</v>
+        <v>opell-prima-020</v>
       </c>
       <c r="C86" t="str">
-        <v>OPELL-PRIMA-021</v>
+        <v>OPELL-PRIMA-023</v>
       </c>
       <c r="D86" t="str">
-        <v>Diverter Body for ALL Colour and Gold Combination</v>
+        <v/>
       </c>
       <c r="E86" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F86" t="str">
-        <v/>
+        <v>Matt Beige</v>
       </c>
       <c r="G86" t="str">
         <v/>
@@ -4677,7 +4677,7 @@
         <v/>
       </c>
       <c r="I86" t="str">
-        <v>opell-prima-021-main.png</v>
+        <v>opell-prima-023-main.png</v>
       </c>
       <c r="J86" t="str">
         <v/>
@@ -4706,13 +4706,13 @@
         <v>Opell Prima</v>
       </c>
       <c r="B87" t="str">
-        <v>opell-prima-024</v>
+        <v>opell-prima-021</v>
       </c>
       <c r="C87" t="str">
-        <v>OPELL-PRIMA-024</v>
+        <v>OPELL-PRIMA-021</v>
       </c>
       <c r="D87" t="str">
-        <v>Diverter Upper Part</v>
+        <v>Diverter Body for ALL Colour and Gold Combination</v>
       </c>
       <c r="E87" t="str">
         <v>Faucets</v>
@@ -4727,7 +4727,7 @@
         <v/>
       </c>
       <c r="I87" t="str">
-        <v>opell-prima-024-main.png</v>
+        <v>opell-prima-021-main.png</v>
       </c>
       <c r="J87" t="str">
         <v/>
@@ -4756,19 +4756,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B88" t="str">
-        <v>opell-prima-025</v>
+        <v>opell-prima-024</v>
       </c>
       <c r="C88" t="str">
-        <v>OPELL-PRIMA-025</v>
+        <v>OPELL-PRIMA-024</v>
       </c>
       <c r="D88" t="str">
-        <v>Diverter Upper Parts</v>
+        <v>Exposed Parts for Single Lever High Flow Diverter Body</v>
       </c>
       <c r="E88" t="str">
         <v>Faucets</v>
       </c>
       <c r="F88" t="str">
-        <v/>
+        <v>Matt Black</v>
       </c>
       <c r="G88" t="str">
         <v/>
@@ -4777,7 +4777,7 @@
         <v/>
       </c>
       <c r="I88" t="str">
-        <v>opell-prima-025-main.png</v>
+        <v>opell-prima-024-main.png</v>
       </c>
       <c r="J88" t="str">
         <v/>
@@ -4806,19 +4806,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B89" t="str">
-        <v>opell-prima-026</v>
+        <v>opell-prima-024</v>
       </c>
       <c r="C89" t="str">
-        <v>OPELL-PRIMA-026</v>
+        <v>OPELL-PRIMA-025</v>
       </c>
       <c r="D89" t="str">
-        <v>Exposed Parts for Single Lever High Flow Diverter Body</v>
+        <v/>
       </c>
       <c r="E89" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F89" t="str">
-        <v/>
+        <v>Rich Gold</v>
       </c>
       <c r="G89" t="str">
         <v/>
@@ -4827,7 +4827,7 @@
         <v/>
       </c>
       <c r="I89" t="str">
-        <v>opell-prima-026-main.jpg</v>
+        <v>opell-prima-025-main.png</v>
       </c>
       <c r="J89" t="str">
         <v/>
@@ -4856,19 +4856,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B90" t="str">
-        <v>opell-prima-027</v>
+        <v>opell-prima-024</v>
       </c>
       <c r="C90" t="str">
-        <v>OPELL-PRIMA-027</v>
+        <v>OPELL-PRIMA-026</v>
       </c>
       <c r="D90" t="str">
-        <v>Gold</v>
+        <v/>
       </c>
       <c r="E90" t="str">
-        <v>Accessories</v>
+        <v/>
       </c>
       <c r="F90" t="str">
-        <v/>
+        <v>Chrome</v>
       </c>
       <c r="G90" t="str">
         <v/>
@@ -4877,7 +4877,7 @@
         <v/>
       </c>
       <c r="I90" t="str">
-        <v>opell-prima-027-main.png</v>
+        <v>opell-prima-026-main.jpg</v>
       </c>
       <c r="J90" t="str">
         <v/>
@@ -4906,16 +4906,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B91" t="str">
-        <v>opell-prima-029</v>
+        <v>opell-prima-027</v>
       </c>
       <c r="C91" t="str">
-        <v>OPELL-PRIMA-029</v>
+        <v>OPELL-PRIMA-027</v>
       </c>
       <c r="D91" t="str">
-        <v>Hand Shower</v>
+        <v>Gold</v>
       </c>
       <c r="E91" t="str">
-        <v>Showers</v>
+        <v>Accessories</v>
       </c>
       <c r="F91" t="str">
         <v/>
@@ -4927,7 +4927,7 @@
         <v/>
       </c>
       <c r="I91" t="str">
-        <v>opell-prima-029-main.png</v>
+        <v>opell-prima-027-main.png</v>
       </c>
       <c r="J91" t="str">
         <v/>
@@ -4959,16 +4959,16 @@
         <v>opell-prima-029</v>
       </c>
       <c r="C92" t="str">
-        <v>OPELL-PRIMA-028</v>
+        <v>OPELL-PRIMA-029</v>
       </c>
       <c r="D92" t="str">
-        <v/>
+        <v>Hand Shower</v>
       </c>
       <c r="E92" t="str">
-        <v/>
+        <v>Showers</v>
       </c>
       <c r="F92" t="str">
-        <v>Rose Gold</v>
+        <v/>
       </c>
       <c r="G92" t="str">
         <v/>
@@ -4977,7 +4977,7 @@
         <v/>
       </c>
       <c r="I92" t="str">
-        <v>opell-prima-028-main.png</v>
+        <v>opell-prima-029-main.png</v>
       </c>
       <c r="J92" t="str">
         <v/>
@@ -5009,7 +5009,7 @@
         <v>opell-prima-029</v>
       </c>
       <c r="C93" t="str">
-        <v>OPELL-PRIMA-030</v>
+        <v>OPELL-PRIMA-028</v>
       </c>
       <c r="D93" t="str">
         <v/>
@@ -5018,7 +5018,7 @@
         <v/>
       </c>
       <c r="F93" t="str">
-        <v>Rich Gold</v>
+        <v>Rose Gold</v>
       </c>
       <c r="G93" t="str">
         <v/>
@@ -5027,7 +5027,7 @@
         <v/>
       </c>
       <c r="I93" t="str">
-        <v>opell-prima-030-main.png</v>
+        <v>opell-prima-028-main.png</v>
       </c>
       <c r="J93" t="str">
         <v/>
@@ -5056,19 +5056,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B94" t="str">
-        <v>opell-prima-031</v>
+        <v>opell-prima-029</v>
       </c>
       <c r="C94" t="str">
-        <v>OPELL-PRIMA-031</v>
+        <v>OPELL-PRIMA-030</v>
       </c>
       <c r="D94" t="str">
-        <v>Health Faucet</v>
+        <v/>
       </c>
       <c r="E94" t="str">
-        <v>Accessories</v>
+        <v/>
       </c>
       <c r="F94" t="str">
-        <v/>
+        <v>Rich Gold</v>
       </c>
       <c r="G94" t="str">
         <v/>
@@ -5077,7 +5077,7 @@
         <v/>
       </c>
       <c r="I94" t="str">
-        <v>opell-prima-031-main.png</v>
+        <v>opell-prima-030-main.png</v>
       </c>
       <c r="J94" t="str">
         <v/>
@@ -5106,16 +5106,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B95" t="str">
-        <v>opell-prima-032</v>
+        <v>opell-prima-031</v>
       </c>
       <c r="C95" t="str">
-        <v>OPELL-PRIMA-032</v>
+        <v>OPELL-PRIMA-031</v>
       </c>
       <c r="D95" t="str">
-        <v>Long Body</v>
+        <v>Health Faucet</v>
       </c>
       <c r="E95" t="str">
-        <v>Faucets</v>
+        <v>Accessories</v>
       </c>
       <c r="F95" t="str">
         <v/>
@@ -5127,7 +5127,7 @@
         <v/>
       </c>
       <c r="I95" t="str">
-        <v>opell-prima-032-main.jpg</v>
+        <v>opell-prima-031-main.png</v>
       </c>
       <c r="J95" t="str">
         <v/>
@@ -5156,16 +5156,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B96" t="str">
-        <v>opell-prima-033</v>
+        <v>opell-prima-032</v>
       </c>
       <c r="C96" t="str">
-        <v>OPELL-PRIMA-033</v>
+        <v>OPELL-PRIMA-032</v>
       </c>
       <c r="D96" t="str">
-        <v>Matte Beige Alive</v>
+        <v>Long Body</v>
       </c>
       <c r="E96" t="str">
-        <v>Accessories</v>
+        <v>Faucets</v>
       </c>
       <c r="F96" t="str">
         <v/>
@@ -5177,7 +5177,7 @@
         <v/>
       </c>
       <c r="I96" t="str">
-        <v>opell-prima-033-main.png</v>
+        <v>opell-prima-032-main.jpg</v>
       </c>
       <c r="J96" t="str">
         <v/>
@@ -5412,13 +5412,13 @@
         <v>OPELL-PRIMA-038</v>
       </c>
       <c r="D101" t="str">
-        <v>Pillar Cock Extend</v>
+        <v>Single Lever Basin Mixer Tall</v>
       </c>
       <c r="E101" t="str">
         <v>Faucets</v>
       </c>
       <c r="F101" t="str">
-        <v/>
+        <v>Matt Beige</v>
       </c>
       <c r="G101" t="str">
         <v/>
@@ -5456,19 +5456,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B102" t="str">
-        <v>opell-prima-039</v>
+        <v>opell-prima-038</v>
       </c>
       <c r="C102" t="str">
         <v>OPELL-PRIMA-039</v>
       </c>
       <c r="D102" t="str">
-        <v>Pillar Cock Extended</v>
+        <v/>
       </c>
       <c r="E102" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F102" t="str">
-        <v/>
+        <v>Rose Gold</v>
       </c>
       <c r="G102" t="str">
         <v/>
@@ -5506,19 +5506,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B103" t="str">
-        <v>opell-prima-040</v>
+        <v>opell-prima-038</v>
       </c>
       <c r="C103" t="str">
-        <v>OPELL-PRIMA-040</v>
+        <v>OPELL-PRIMA-048</v>
       </c>
       <c r="D103" t="str">
-        <v>Pillar Cock Extended Body</v>
+        <v/>
       </c>
       <c r="E103" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F103" t="str">
-        <v/>
+        <v>Chrome</v>
       </c>
       <c r="G103" t="str">
         <v/>
@@ -5527,7 +5527,7 @@
         <v/>
       </c>
       <c r="I103" t="str">
-        <v>opell-prima-040-main.jpg</v>
+        <v>opell-prima-048-main.jpg</v>
       </c>
       <c r="J103" t="str">
         <v/>
@@ -5556,19 +5556,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B104" t="str">
-        <v>opell-prima-041</v>
+        <v>opell-prima-038</v>
       </c>
       <c r="C104" t="str">
-        <v>OPELL-PRIMA-041</v>
+        <v>OPELL-PRIMA-049</v>
       </c>
       <c r="D104" t="str">
-        <v>Plain Spout</v>
+        <v/>
       </c>
       <c r="E104" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F104" t="str">
-        <v/>
+        <v>Matt White</v>
       </c>
       <c r="G104" t="str">
         <v/>
@@ -5577,7 +5577,7 @@
         <v/>
       </c>
       <c r="I104" t="str">
-        <v>opell-prima-041-main.png</v>
+        <v>opell-prima-049-main.png</v>
       </c>
       <c r="J104" t="str">
         <v/>
@@ -5606,19 +5606,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B105" t="str">
-        <v>opell-prima-042</v>
+        <v>opell-prima-038</v>
       </c>
       <c r="C105" t="str">
-        <v>OPELL-PRIMA-042</v>
+        <v>OPELL-PRIMA-050</v>
       </c>
       <c r="D105" t="str">
-        <v>Shower ARM</v>
+        <v/>
       </c>
       <c r="E105" t="str">
-        <v>Showers</v>
+        <v/>
       </c>
       <c r="F105" t="str">
-        <v/>
+        <v>Matt Beige Gold</v>
       </c>
       <c r="G105" t="str">
         <v/>
@@ -5627,7 +5627,7 @@
         <v/>
       </c>
       <c r="I105" t="str">
-        <v>opell-prima-042-main.png</v>
+        <v>opell-prima-050-main.png</v>
       </c>
       <c r="J105" t="str">
         <v/>
@@ -5656,19 +5656,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B106" t="str">
-        <v>opell-prima-042</v>
+        <v>opell-prima-040</v>
       </c>
       <c r="C106" t="str">
-        <v>OPELL-PRIMA-043</v>
+        <v>OPELL-PRIMA-040</v>
       </c>
       <c r="D106" t="str">
-        <v/>
+        <v>Pillar Cock Extended Body</v>
       </c>
       <c r="E106" t="str">
-        <v/>
+        <v>Faucets</v>
       </c>
       <c r="F106" t="str">
-        <v>Matt Black Gold</v>
+        <v/>
       </c>
       <c r="G106" t="str">
         <v/>
@@ -5677,7 +5677,7 @@
         <v/>
       </c>
       <c r="I106" t="str">
-        <v>opell-prima-043-main.png</v>
+        <v>opell-prima-040-main.jpg</v>
       </c>
       <c r="J106" t="str">
         <v/>
@@ -5706,16 +5706,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B107" t="str">
-        <v>opell-prima-044</v>
+        <v>opell-prima-041</v>
       </c>
       <c r="C107" t="str">
-        <v>OPELL-PRIMA-044</v>
+        <v>OPELL-PRIMA-041</v>
       </c>
       <c r="D107" t="str">
-        <v>Shower Head</v>
+        <v>Plain Spout</v>
       </c>
       <c r="E107" t="str">
-        <v>Showers</v>
+        <v>Faucets</v>
       </c>
       <c r="F107" t="str">
         <v/>
@@ -5727,7 +5727,7 @@
         <v/>
       </c>
       <c r="I107" t="str">
-        <v>opell-prima-044-main.png</v>
+        <v>opell-prima-041-main.png</v>
       </c>
       <c r="J107" t="str">
         <v/>
@@ -5756,19 +5756,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B108" t="str">
-        <v>opell-prima-044</v>
+        <v>opell-prima-042</v>
       </c>
       <c r="C108" t="str">
-        <v>OPELL-PRIMA-045</v>
+        <v>OPELL-PRIMA-042</v>
       </c>
       <c r="D108" t="str">
-        <v/>
+        <v>Shower ARM</v>
       </c>
       <c r="E108" t="str">
-        <v/>
+        <v>Showers</v>
       </c>
       <c r="F108" t="str">
-        <v>Matt Beige</v>
+        <v/>
       </c>
       <c r="G108" t="str">
         <v/>
@@ -5777,7 +5777,7 @@
         <v/>
       </c>
       <c r="I108" t="str">
-        <v>opell-prima-045-main.png</v>
+        <v>opell-prima-042-main.png</v>
       </c>
       <c r="J108" t="str">
         <v/>
@@ -5806,19 +5806,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B109" t="str">
-        <v>opell-prima-046</v>
+        <v>opell-prima-042</v>
       </c>
       <c r="C109" t="str">
-        <v>OPELL-PRIMA-046</v>
+        <v>OPELL-PRIMA-043</v>
       </c>
       <c r="D109" t="str">
-        <v>Shower Mixer for Spout Only</v>
+        <v/>
       </c>
       <c r="E109" t="str">
-        <v>Showers</v>
+        <v/>
       </c>
       <c r="F109" t="str">
-        <v/>
+        <v>Matt Black Gold</v>
       </c>
       <c r="G109" t="str">
         <v/>
@@ -5827,7 +5827,7 @@
         <v/>
       </c>
       <c r="I109" t="str">
-        <v>opell-prima-046-main.jpg</v>
+        <v>opell-prima-043-main.png</v>
       </c>
       <c r="J109" t="str">
         <v/>
@@ -5856,16 +5856,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B110" t="str">
-        <v>opell-prima-047</v>
+        <v>opell-prima-044</v>
       </c>
       <c r="C110" t="str">
-        <v>OPELL-PRIMA-047</v>
+        <v>OPELL-PRIMA-044</v>
       </c>
       <c r="D110" t="str">
-        <v>Single Lever Basin Mixer</v>
+        <v>Shower Head</v>
       </c>
       <c r="E110" t="str">
-        <v>Faucets</v>
+        <v>Showers</v>
       </c>
       <c r="F110" t="str">
         <v/>
@@ -5877,10 +5877,10 @@
         <v/>
       </c>
       <c r="I110" t="str">
-        <v>opell-prima-047-main.jpg</v>
+        <v>opell-prima-044-main.png</v>
       </c>
       <c r="J110" t="str">
-        <v>opell-prima-047-main.jpg,opell-prima-059-main.png</v>
+        <v/>
       </c>
       <c r="K110" t="str">
         <v/>
@@ -5906,19 +5906,19 @@
         <v>Opell Prima</v>
       </c>
       <c r="B111" t="str">
-        <v>opell-prima-048</v>
+        <v>opell-prima-044</v>
       </c>
       <c r="C111" t="str">
-        <v>OPELL-PRIMA-048</v>
+        <v>OPELL-PRIMA-045</v>
       </c>
       <c r="D111" t="str">
-        <v>Single Lever Basin Mixer Extended Body</v>
+        <v/>
       </c>
       <c r="E111" t="str">
-        <v>Faucets</v>
+        <v/>
       </c>
       <c r="F111" t="str">
-        <v/>
+        <v>Matt Beige</v>
       </c>
       <c r="G111" t="str">
         <v/>
@@ -5927,7 +5927,7 @@
         <v/>
       </c>
       <c r="I111" t="str">
-        <v>opell-prima-048-main.jpg</v>
+        <v>opell-prima-045-main.png</v>
       </c>
       <c r="J111" t="str">
         <v/>
@@ -5956,16 +5956,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B112" t="str">
-        <v>opell-prima-049</v>
+        <v>opell-prima-046</v>
       </c>
       <c r="C112" t="str">
-        <v>OPELL-PRIMA-049</v>
+        <v>OPELL-PRIMA-046</v>
       </c>
       <c r="D112" t="str">
-        <v>Single Lever Basin Mixer Tall</v>
+        <v>Shower Mixer for Spout Only</v>
       </c>
       <c r="E112" t="str">
-        <v>Faucets</v>
+        <v>Showers</v>
       </c>
       <c r="F112" t="str">
         <v/>
@@ -5977,10 +5977,10 @@
         <v/>
       </c>
       <c r="I112" t="str">
-        <v>opell-prima-049-main.png</v>
+        <v>opell-prima-046-main.jpg</v>
       </c>
       <c r="J112" t="str">
-        <v>opell-prima-049-main.png,opell-prima-060-main.png</v>
+        <v/>
       </c>
       <c r="K112" t="str">
         <v/>
@@ -6006,16 +6006,16 @@
         <v>Opell Prima</v>
       </c>
       <c r="B113" t="str">
-        <v>opell-prima-050</v>
+        <v>opell-prima-047</v>
       </c>
       <c r="C113" t="str">
-        <v>OPELL-PRIMA-050</v>
+        <v>OPELL-PRIMA-047</v>
       </c>
       <c r="D113" t="str">
-        <v>Single Lever Basin Tall</v>
+        <v>Single Lever Basin Mixer</v>
       </c>
       <c r="E113" t="str">
-        <v>Accessories</v>
+        <v>Faucets</v>
       </c>
       <c r="F113" t="str">
         <v/>
@@ -6027,10 +6027,10 @@
         <v/>
       </c>
       <c r="I113" t="str">
-        <v>opell-prima-050-main.png</v>
+        <v>opell-prima-047-main.jpg</v>
       </c>
       <c r="J113" t="str">
-        <v/>
+        <v>opell-prima-047-main.jpg,opell-prima-059-main.png</v>
       </c>
       <c r="K113" t="str">
         <v/>

</xml_diff>